<commit_message>
Update binary files for CournotCompetition figures and data
</commit_message>
<xml_diff>
--- a/CournotCompetition/figs/total_revenue.xlsx
+++ b/CournotCompetition/figs/total_revenue.xlsx
@@ -517,22 +517,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>126097949469 $\pm$ 5599135398</t>
+          <t>613457758794 $\pm$ 3207538001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>111442361129 $\pm$ 6489275657</t>
+          <t>553653601740 $\pm$ 4253940560</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>99211826774 $\pm$ 5008231589</t>
+          <t>495873467847 $\pm$ 3374417934</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>85652192032 $\pm$ 4706298627</t>
+          <t>432605102061 $\pm$ 2661304876</t>
         </is>
       </c>
     </row>
@@ -544,22 +544,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>541632808959 $\pm$ 4252484004</t>
+          <t>614550589246 $\pm$ 3829250792</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>474017026759 $\pm$ 5524736995</t>
+          <t>552457593235 $\pm$ 4741244927</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>412973023963 $\pm$ 3675382710</t>
+          <t>494733428903 $\pm$ 3517588370</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>353327252448 $\pm$ 4286103724</t>
+          <t>434933680908 $\pm$ 4873485422</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor gradient calculation in runRGD and runSFB functions for improved accuracy; update binary output files for figures and data
</commit_message>
<xml_diff>
--- a/CournotCompetition/figs/total_revenue.xlsx
+++ b/CournotCompetition/figs/total_revenue.xlsx
@@ -517,22 +517,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>613457758794 $\pm$ 3207538001</t>
+          <t>126097949469 $\pm$ 5599135398</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>553653601740 $\pm$ 4253940560</t>
+          <t>111442361129 $\pm$ 6489275657</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>495873467847 $\pm$ 3374417934</t>
+          <t>99211826774 $\pm$ 5008231589</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>432605102061 $\pm$ 2661304876</t>
+          <t>85652192032 $\pm$ 4706298627</t>
         </is>
       </c>
     </row>
@@ -544,22 +544,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>614550589246 $\pm$ 3829250792</t>
+          <t>541632808959 $\pm$ 4252484004</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>552457593235 $\pm$ 4741244927</t>
+          <t>474017026759 $\pm$ 5524736995</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>494733428903 $\pm$ 3517588370</t>
+          <t>412973023963 $\pm$ 3675382710</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>434933680908 $\pm$ 4873485422</t>
+          <t>353327252448 $\pm$ 4286103724</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update initial point range, refine gradient calculations, and enhance plotting for revenue and quantity variations; update binary output files accordingly
</commit_message>
<xml_diff>
--- a/CournotCompetition/figs/total_revenue.xlsx
+++ b/CournotCompetition/figs/total_revenue.xlsx
@@ -517,22 +517,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>111162466311 $\pm$ 1514598367</t>
+          <t>118313395016 $\pm$ 867566985</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>97967355550 $\pm$ 1107309184</t>
+          <t>104466540145 $\pm$ 645281801</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>85844124129 $\pm$ 1719108614</t>
+          <t>91690507635 $\pm$ 993368768</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>72355313726 $\pm$ 1487809155</t>
+          <t>78509390697 $\pm$ 835770396</t>
         </is>
       </c>
     </row>
@@ -544,22 +544,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>203984442314 $\pm$ 7216682775</t>
+          <t>235378270288 $\pm$ 4187677120</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>167956191740 $\pm$ 5236006687</t>
+          <t>197475481461 $\pm$ 2969661817</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>134883303314 $\pm$ 8478914306</t>
+          <t>162490825267 $\pm$ 4876880178</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>93022810478 $\pm$ 8070299844</t>
+          <t>123608760492 $\pm$ 4656565976</t>
         </is>
       </c>
     </row>
@@ -571,22 +571,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>-215789421540 $\pm$ 999602121696</t>
+          <t>159323190515 $\pm$ 284340602825</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>-1184297763397 $\pm$ 3317469030083</t>
+          <t>310759377382 $\pm$ 131386077906</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-5341467434809 $\pm$ 14424516229194</t>
+          <t>71846217891 $\pm$ 186332867822</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>-1377050782057 $\pm$ 3514342444889</t>
+          <t>202309793799 $\pm$ 185242187655</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor model list and update run functions for improved accuracy; add runRR method for repeated retraining in ride share module
</commit_message>
<xml_diff>
--- a/CournotCompetition/figs/total_revenue.xlsx
+++ b/CournotCompetition/figs/total_revenue.xlsx
@@ -598,22 +598,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>297212091100 $\pm$ 54457366832</t>
+          <t>361785347443 $\pm$ 68669589294</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>233505327608 $\pm$ 75972292809</t>
+          <t>355973349480 $\pm$ 36688804447</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>181244146006 $\pm$ 60056530193</t>
+          <t>281432972894 $\pm$ 89134716146</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>85106284879 $\pm$ 77867494204</t>
+          <t>208427770814 $\pm$ 69948415659</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update learning rate in synthetic strategic prediction for improved stability
</commit_message>
<xml_diff>
--- a/CournotCompetition/figs/total_revenue.xlsx
+++ b/CournotCompetition/figs/total_revenue.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -571,49 +571,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>433208230449 $\pm$ 105572359726</t>
+          <t>433459478716 $\pm$ 105348939269</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>449949559027 $\pm$ 93492000718</t>
+          <t>449946660353 $\pm$ 93499995514</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>275710029581 $\pm$ 147699664386</t>
+          <t>275708975998 $\pm$ 147699583764</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>234503382649 $\pm$ 190568312791</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>OPGD</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>361785347443 $\pm$ 68669589294</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>355973349480 $\pm$ 36688804447</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>281432972894 $\pm$ 89134716146</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>208427770814 $\pm$ 69948415659</t>
+          <t>237023914683 $\pm$ 190200297926</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor titles in plots and update labels for clarity in Cournot competition analysis
</commit_message>
<xml_diff>
--- a/CournotCompetition/figs/total_revenue.xlsx
+++ b/CournotCompetition/figs/total_revenue.xlsx
@@ -436,22 +436,22 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>$\mu_A$ = 0.25</t>
+          <t>$\mu$ = 0.25</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>$\mu_A$ = 0.5</t>
+          <t>$\mu$ = 0.5</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>$\mu_A$ = 0.75</t>
+          <t>$\mu$ = 0.75</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>$\mu_A$ = 1.0</t>
+          <t>$\mu$ = 1.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update experiment configuration and enhance plot labels for clarity in Cournot competition analysis
</commit_message>
<xml_diff>
--- a/CournotCompetition/figs/total_revenue.xlsx
+++ b/CournotCompetition/figs/total_revenue.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -587,6 +587,33 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>237023914683 $\pm$ 190200297926</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>OPGD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>361785347443 $\pm$ 68669589294</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>355973349480 $\pm$ 36688804447</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>281432972894 $\pm$ 89134716146</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>208427770814 $\pm$ 69948415659</t>
         </is>
       </c>
     </row>

</xml_diff>